<commit_message>
Update workbench screening workflow
</commit_message>
<xml_diff>
--- a/有道答疑笔5-6月合作_测试项目/有道答疑笔5-6月合作_测试项目.xlsx
+++ b/有道答疑笔5-6月合作_测试项目/有道答疑笔5-6月合作_测试项目.xlsx
@@ -2194,31 +2194,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y11"/>
+  <dimension ref="A1:AD24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.72727272727273" defaultRowHeight="14"/>
   <cols>
-    <col width="8.54545454545454" customWidth="1" style="3" min="1" max="1"/>
-    <col width="9.90909090909091" customWidth="1" style="3" min="2" max="2"/>
-    <col width="12.2727272727273" customWidth="1" style="3" min="3" max="3"/>
-    <col width="17.3636363636364" customWidth="1" style="3" min="4" max="4"/>
-    <col width="19.6363636363636" customWidth="1" style="3" min="5" max="5"/>
-    <col width="15.1818181818182" customWidth="1" style="3" min="6" max="6"/>
-    <col width="5.72727272727273" customWidth="1" style="3" min="7" max="7"/>
-    <col width="9.90909090909091" customWidth="1" style="3" min="8" max="8"/>
-    <col width="14.6363636363636" customWidth="1" style="3" min="9" max="9"/>
-    <col width="7.81818181818182" customWidth="1" style="3" min="10" max="10"/>
-    <col width="19.4545454545455" customWidth="1" style="3" min="11" max="11"/>
-    <col width="14.6363636363636" customWidth="1" style="3" min="12" max="12"/>
-    <col width="18.3636363636364" customWidth="1" style="3" min="13" max="14"/>
-    <col width="15.9090909090909" customWidth="1" style="3" min="15" max="15"/>
-    <col width="19.4545454545455" customWidth="1" style="3" min="16" max="16"/>
-    <col width="9.90909090909091" customWidth="1" style="3" min="17" max="17"/>
-    <col width="23" customWidth="1" style="3" min="18" max="18"/>
-    <col width="9.90909090909091" customWidth="1" style="3" min="19" max="19"/>
-    <col width="32" customWidth="1" style="3" min="20" max="20"/>
-    <col width="19.4545454545455" customWidth="1" style="3" min="21" max="22"/>
-    <col width="9.90909090909091" customWidth="1" style="3" min="23" max="24"/>
-    <col width="15.1818181818182" customWidth="1" style="3" min="25" max="25"/>
+    <col width="40" customWidth="1" style="3" min="1" max="1"/>
+    <col width="12" customWidth="1" style="3" min="2" max="2"/>
+    <col width="40" customWidth="1" style="3" min="3" max="3"/>
+    <col width="10" customWidth="1" style="3" min="4" max="4"/>
+    <col width="27" customWidth="1" style="3" min="5" max="5"/>
+    <col width="11" customWidth="1" style="3" min="6" max="6"/>
+    <col width="10" customWidth="1" style="3" min="7" max="7"/>
+    <col width="10" customWidth="1" style="3" min="8" max="8"/>
+    <col width="10" customWidth="1" style="3" min="9" max="9"/>
+    <col width="10" customWidth="1" style="3" min="10" max="10"/>
+    <col width="11" customWidth="1" style="3" min="11" max="11"/>
+    <col width="10" customWidth="1" style="3" min="12" max="12"/>
+    <col width="11" customWidth="1" style="3" min="13" max="14"/>
+    <col width="11" customWidth="1" style="3" min="14" max="14"/>
+    <col width="10" customWidth="1" style="3" min="15" max="15"/>
+    <col width="11" customWidth="1" style="3" min="16" max="16"/>
+    <col width="10" customWidth="1" style="3" min="17" max="17"/>
+    <col width="10" customWidth="1" style="3" min="18" max="18"/>
+    <col width="10" customWidth="1" style="3" min="19" max="19"/>
+    <col width="14" customWidth="1" style="3" min="20" max="20"/>
+    <col width="11" customWidth="1" style="3" min="21" max="22"/>
+    <col width="11" customWidth="1" style="3" min="22" max="22"/>
+    <col width="10" customWidth="1" style="3" min="23" max="24"/>
+    <col width="10" customWidth="1" style="3" min="24" max="24"/>
+    <col width="10" customWidth="1" style="3" min="25" max="25"/>
+    <col width="10" customWidth="1" style="3" min="26" max="26"/>
+    <col width="10" customWidth="1" style="3" min="27" max="27"/>
+    <col width="10" customWidth="1" style="3" min="28" max="28"/>
+    <col width="40" customWidth="1" style="3" min="29" max="29"/>
+    <col width="40" customWidth="1" style="3" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="2">
@@ -2334,15 +2342,40 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
+          <t>评分总分</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>评分等级</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>推荐等级</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>硬性条件通过</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>达人池分组</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
         <is>
           <t>当前状态</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>合作方向</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -2351,27 +2384,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>KOL-001</t>
+          <t>pgy:朝阳小北妈妈:57000.0:4900.0:北京</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>北京海淀安安妈</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/KOL-001</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>曝光型</t>
-        </is>
-      </c>
+          <t>朝阳小北妈妈</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>高知家庭/亲子大孩</t>
+          <t>6-12岁/妈妈/教育/vlog/教育/教育</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2379,1242 +2404,2002 @@
           <t>北京</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>16800</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>186000</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>稳定</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1.78</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>12.6</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>52%</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>58%</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>小升初</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>女</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>海淀小升初规划、学区房家庭学习效率场景</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
+      <c r="G2" t="n">
+        <v>4900</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="n">
+        <v>57000</v>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="n">
+        <v>86</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>初筛通过</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>曝光型核心候选，家庭叙事贴合答疑笔使用场景</t>
+          <t>推荐</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>待建联达人</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>待补数据</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>适合北京家庭教育焦虑、升学陪伴、晚间答疑提效等场景化内容</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>【大模型分析】北京IP高度契合，教育vlog家庭叙事适合项目，中产家长视角有潜力；但互动中位偏一般，孩子年级、35+粉占比、CPE/CPC、搜索推荐、限流风险和蒲公英链接待补，链接缺失暂未过硬筛。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>KOL-002</t>
+          <t>pgy:Levi爸爸说育儿:20000.0:2000.0:福建 福州 马尾区</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>上海中产陪读日记</t>
+          <t>Levi爸爸说育儿</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/KOL-002</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>曝光型</t>
-        </is>
-      </c>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/64029398000000001001ec3d?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>中产家庭/亲子大孩</t>
+          <t>爸爸/萌娃/教育/母婴/教育/教育</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>上海</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>15200</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>142000</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>稳定</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>1.92</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>14.8</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>48%</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>55%</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>初二</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>男</t>
-        </is>
-      </c>
+          <t>福建 福州 马尾区</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>上海中产教育日常、晚自习陪伴和错题整理</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+          <t>母婴、萌娃、家居家装</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="n">
+        <v>83</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>初筛通过</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>内容真实感强，适合做家庭使用体验笔记</t>
+          <t>备选</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>待建联达人</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>可走爸爸视角家庭学习管理/亲子作业冲突解决内容，适合做讨论型曝光或低成本测试位。</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>【大模型分析】爸爸育儿人设有差异化，报价低但阅读体量高，潜在CPE表现优；不过粉丝年龄显示25-34为主，35+硬性比例需重点补采，孩子阶段也未见初高中明确信号，存在受众错配风险。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KOL-003</t>
+          <t>pgy:硕士奶爸挖宝记:28000.0:3800.0:福建 福州 马尾区</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>胡同里养娃的林老师</t>
+          <t>硕士奶爸挖宝记</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/KOL-003</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>曝光型</t>
-        </is>
-      </c>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/6588fd8d000000001c0284f7?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>教师人设/普通有娃家庭</t>
+          <t>爸爸/萌娃/教育/母婴/开箱/教育/教育</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>北京</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>12600</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>98000</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>稳定</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>1.65</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>9.8</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>57%</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>62%</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>初三</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>女</t>
-        </is>
-      </c>
+          <t>福建 福州 马尾区</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>3800</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>28000</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>教师妈妈视角、胡同家庭备考冲刺和学习工具选择</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
+          <t>母婴、萌娃、家居家装</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="n">
+        <v>83</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>初筛通过</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>教师+家长双人设，话题度高</t>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>待建联达人</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>可做高知爸爸视角的学习工具种草，但仅适合作为观察样本，不建议进入本项目正式合作池。</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>【大模型分析】硕士奶爸、高知家庭与教育场景匹配，报价低且流量表现强；但粉丝年龄25-34占84.1%，已明显不符35岁以上占比＞40%的硬门槛。待补CPC/CPE、搜索推荐占比、孩子年级。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KOL-004</t>
+          <t>pgy:清华丸子雨学姐:45000.0:3500.0:北京</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>住校生妈妈手记</t>
+          <t>清华丸子雨学姐</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/KOL-004</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>曝光型</t>
-        </is>
-      </c>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/5f2a1c4d0000000001000279?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>亲子大孩/普通有娃家庭</t>
+          <t>创业者/学生/教育/vlog/教育/教育</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>上海</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>9800</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>76000</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>波动</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>16.5</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>44%</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>49%</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>高一</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>男</t>
-        </is>
-      </c>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>45000</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>住校生学习自主管理、周末复盘和答疑需求</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+          <t>生活记录、二次元、娱乐</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="n">
+        <v>82</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
           <t>备选</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>CPC略高但人设场景稀缺，可作为备选</t>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>待建联达人</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>可做高知学习方法/家长视角教育工具种草，作为曝光型补位，主打北京高知氛围与学习效率场景。</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>【大模型分析】北京IP、清华学姐高知人设契合，报价低且流量互动不错；但粉丝35+占比、CPC/CPE、搜索推荐占比、孩子阶段均待补，当前受众兴趣偏生活娱乐，需核验是否偏离教育家长人群。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>KOL-005</t>
+          <t>pgy:Peter妈妈:17000.0:2200.0:湖南 株洲 天元区</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>国际学校转轨妈妈</t>
+          <t>Peter妈妈</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/KOL-005</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>曝光型</t>
-        </is>
-      </c>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/5676d41db8ce1a042f292b51?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>高知家庭/中产家庭</t>
+          <t>6-12岁/妈妈/教育/母婴/3+/教育/教育</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>上海</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>18800</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>231000</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>稳定</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>1.88</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>46%</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>53%</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>初一</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>女</t>
-        </is>
-      </c>
+          <t>湖南 株洲 天元区</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="n">
+        <v>17000</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>国际学校转轨、英语学习和课后答疑陪伴</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+          <t>母婴、教育、美食</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="n">
+        <v>79</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>初筛通过</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>需复核近期争议内容，预算内可推进</t>
+          <t>备选</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>待建联达人</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>适合普通有娃家庭学习场景，主打家长陪学、作业答疑、家庭教育工具实用种草。</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>【大模型分析】妈妈+教育母婴场景匹配，报价低、互动和增长表现尚可；但孩子年级未明确，35岁+粉丝占比、CPC/CPE、搜索推荐占比均待补，且非北上IP。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KOL-006</t>
+          <t>pgy:嘟嘟仔:13000.0:4200.0:浙江 台州 温岭市</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>初中数学周老师</t>
+          <t>嘟嘟仔</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/KOL-006</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>教育垂类/卖货型</t>
-        </is>
-      </c>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/55faaeb341a2b34bcee5d724?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>教师人设/初高中学习陪伴</t>
+          <t>6-12岁/妈妈/教育/母婴/开箱/教育/教育</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>北京</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>13600</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>164000</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>稳定</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>1.42</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>8.6</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>61%</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>64%</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>初一</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>未披露</t>
-        </is>
-      </c>
+          <t>浙江 台州 温岭市</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>4200</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>13000</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>数学学习方法、错题本和课后答疑工具推荐</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
+          <t>母婴、萌娃、家居家装</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="n">
+        <v>78</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>初筛通过</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>教育垂类转化基础好，优先沟通</t>
+          <t>备选</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>待建联达人</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>可走家长陪学、作业辅导、学习习惯培养方向，作为教育/亲子腰尾部补位达人。</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>【大模型分析】6-12岁妈妈且带教育标签，内容场景与学习工具较匹配，报价可控；但粉丝35+、CPC/CPE、搜索推荐占比均缺失，孩子是否小升初/初高中待补，地域非京沪。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>KOL-007</t>
+          <t>pgy:S-L-Y酸辣鱼:12000.0:1600.0:辽宁 沈阳 沈河区</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>升学政策研究员Grace</t>
+          <t>S-L-Y酸辣鱼</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/KOL-007</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>教育垂类/卖货型</t>
-        </is>
-      </c>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/5f0500660000000001002622?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>教育政策解读/高知教育达人</t>
+          <t>6-12岁/妈妈/教育/母婴/教程/教育/教育</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>北京</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>17800</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>205000</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>稳定</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>1.70</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>11.4</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>55%</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>67%</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>小升初</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>未披露</t>
-        </is>
-      </c>
+          <t>辽宁 沈阳 沈河区</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1600</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="n">
+        <v>12000</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>升学政策、学习规划和家长决策链路</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
+          <t>母婴、萌娃、家居家装</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="n">
+        <v>76</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>初筛通过</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>35岁以上粉丝占比高，适合承接家长搜索需求</t>
+          <t>备选</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>待建联达人</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>适合家长辅导痛点、作业检查、家庭学习管理等实用型种草，偏性价比补位。</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>【大模型分析】6-12岁妈妈+教育母婴教程，内容场景可承接答疑笔，报价极优；但孩子是否小升初/初高中未明，35岁+粉丝占比、CPE/CPC、搜索推荐占比待补，非北上IP。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KOL-008</t>
+          <t>pgy:京妈说:13000.0:2500.0:天津</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>陪娃刷题的陈博士</t>
+          <t>京妈说</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/KOL-008</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>教育垂类/卖货型</t>
-        </is>
-      </c>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/556cd2ede58d131daeb485e9?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>高知家庭/高知教育达人</t>
+          <t>6-12岁/妈妈/教育/母婴/测评/教育/教育</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>上海</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>16500</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>119000</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>稳定</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>1.56</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>9.2</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>59%</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>60%</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>高二</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>男</t>
-        </is>
-      </c>
+          <t>天津</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>13000</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>理工科家长陪读、理科答疑和学习效率工具</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
+          <t>母婴、家居家装、萌娃</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="n">
+        <v>76</v>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>初筛通过</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>专业信任感强，适合答疑笔功能深度种草</t>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>待建联达人</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>若后续粉丝年龄核验达标，可尝试妈妈视角的学习辅导场景测评；当前不建议优先推进。</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>【大模型分析】教育母婴妈妈人设、报价低、互动率高，具一定种草效率；但粉丝年龄仅知25-34占49.7%，无法支持35岁以上占比＞40%，按硬筛倾向不通过。待补孩子阶段、CPC/CPE、搜索推荐占比。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KOL-009</t>
+          <t>pgy:Julia生活育儿:23000.0:2900.0:陕西 西安 碑林区</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>教辅工具测评小乔</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/KOL-009</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>教育垂类/卖货型</t>
-        </is>
-      </c>
+          <t>Julia生活育儿</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>亲子教育卖货型/学习用品</t>
+          <t>6-12岁/妈妈/教育/母婴/2+/教育/教育</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>8200</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>68000</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>稳定</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>1.35</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>7.9</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>63%</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>46%</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>初二</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>女</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>学习用品横评、教辅工具对比和真实转化复盘</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+          <t>陕西 西安 碑林区</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>2900</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>23000</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="n">
+        <v>75</v>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>初筛通过</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>非京沪但数据效率优秀，可补足卖货型结构</t>
+          <t>备选</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>待建联达人</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>待补数据</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>适合家长陪学、作业订正、知识点答疑工具测评与日常学习vlog</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>【大模型分析】阅读互动中位数尚可，教育母婴内容具备植入空间，报价低；但城市非优先，孩子阶段仅6-12岁偏泛，35+粉占比、自然流量效率、搜索推荐、限流风险及蒲公英链接待补，需补证后判断。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>KOL-010</t>
+          <t>pgy:爱学习的可乐🥤:8400.0:1850.0:安徽 合肥 包河区</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>高中陪跑老爸</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/KOL-010</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>教育垂类/卖货型</t>
-        </is>
-      </c>
+          <t>爱学习的可乐🥤</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>初高中学习陪伴/普通有娃家庭</t>
+          <t>6-12岁/萌娃/教育/测评/vlog/教育/教育</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>北京</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>11200</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>87000</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>波动</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>1.84</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>10.6</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>51%</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>高三</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>男</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>高三复习陪跑、家长情绪管理和即时答疑需求</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
+          <t>安徽 合肥 包河区</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1850</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>8400</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="n">
+        <v>72</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>备选</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>待建联达人</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>待补数据</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>适合做学习工具测评、作业辅导场景种草，偏性价比补位账号</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>【大模型分析】报价低、教育测评vlog可植入，但孩子仅见6-12岁，偏小学段；35+粉占比、CPC/CPE、搜索推荐占比、限流风险与蒲公英链接均待补，且链接缺失触发硬性项。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>pgy:金豆妈爱分享:16000.0:2500.0:江苏 徐州 泉山区</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Julia生活育儿</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/668cc4d6000000000b03186b?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>6-12岁/妈妈/教育/母婴/2+/教育/教育</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>陕西 西安 碑林区</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>2900</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>23000</v>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>41%</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>母婴、美食、家居家装</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="n">
+        <v>90</v>
+      </c>
+      <c r="X12" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>初筛通过</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>男性家长视角有差异化，注意排期接近尾段</t>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>推荐</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>已驳回</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>适合家长真实陪学、家庭作业辅导、孩子学习效率提升等场景，作为教育母婴种草型达人优先补采。</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>【大模型分析】妈妈+教育母婴人设契合，粉丝35-44占41.3%满足硬门槛，报价低、粉丝活跃和增速不错；但孩子年级、CPC/CPE、搜索推荐占比、限流风险仍待补，且非京沪IP略减分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>pgy:爱动手的Betty妈:20000.0:3000.0:福建 厦门 同安区</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>爱动手的Betty妈</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>6-12岁/妈妈/教育/母婴/2+/教育/教育</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>福建 厦门 同安区</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="n">
+        <v>20000</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="n">
+        <v>69</v>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>待补数据</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>若补证孩子临近升学，可尝试家长陪学、作业管理类轻种草内容</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>【大模型分析】报价友好，教育母婴妈妈有一定相关性，但更偏6-12岁泛育儿，缺少初高中/小升初信号；35+粉占比、自然流量效率、搜索推荐、限流风险、蒲公英链接待补，当前不宜优先。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>pgy:可慕妈妈:11000.0:1700.0:吉林 长春 南关区</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>可慕妈妈</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>6-12岁/萌娃/教育/母婴/3+/教育/教育</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>吉林 长春 南关区</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1700</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="n">
+        <v>11000</v>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>64</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>已驳回</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>如后续补齐链接与核心数据，可尝试小学高年级学习工具种草，但当前不进入主池。</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>【大模型分析】教育母婴标签和6-12岁阶段有一定相关性，且报价低；但缺少蒲公英链接已触发硬性不符，粉丝年龄、CPC/CPE、流量来源等关键信息缺失，孩子年级也未明确。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>pgy:妤熙麻麻:13000.0:1500.0:重庆</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>妤熙麻麻</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/5a8069a7e8ac2b6ad96808f0?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>6-12岁/萌娃/教育/母婴/vlog/教育/教育</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="n">
+        <v>13000</v>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>母婴、萌娃、家居家装</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="n">
+        <v>63</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>如补证孩子已到高年级，可尝试家庭作业辅导/学习效率工具种草；更适合作为低成本长尾备选。</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>【大模型分析】有蒲公英链接、报价低，教育母婴场景可植入；但孩子更像6-12岁，未见初高中大孩信号，且粉丝35+占比、CPC/CPE、搜索推荐占比与流量数据缺失较多，项目适配度偏弱。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>pgy:Lolaaaa:51000.0:4500.0:上海</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Lolaaaa</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>学生/教育/plog/2+/教育/教育</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>4500</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="n">
+        <v>51000</v>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="n">
+        <v>60</v>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>待补数据</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>更适合学生自用或校园内容，不适合本次家长教育决策型项目投放。</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>【大模型分析】上海IP有加分，报价也低；但学生人设与项目核心的家长/教师/高知家庭不匹配，且缺失蒲公英链接，命中硬性要求。粉丝画像、效率、流量稳定性均待补，当前不具备推进价值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>pgy:小狮子当当:27000.0:2500.0:四川 成都 双流区</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>小狮子当当</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>6-12岁/萌娃/教育/母婴/3+/教育/教育</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>四川 成都 双流区</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>2500</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="n">
+        <v>27000</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="n">
+        <v>58</v>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>待补数据</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>若后续补齐链接且孩子已进入高年级，可再看家庭学习陪伴类；当前不建议进入本项目。</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>【大模型分析】缺少蒲公英链接，命中硬性项；且现有人设偏6-12岁萌娃母婴，不是小升初/初高中大孩方向。报价低但核心受众、孩子阶段、35+占比及成本效率均未证实。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>pgy:依依有个姐姐:45000.0:2000.0:山西 太原 小店区</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>依依有个姐姐</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/604eaa5400000000010007aa?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>学生/家庭/教育/vlog/沉浸式/教育/教育</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>山西 太原 小店区</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="n">
+        <v>45000</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>生活记录、教育、娱乐</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="n">
+        <v>54</v>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>更适合学生学习效率或校园内容，不适合本项目核心家长决策人群投放。</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>【大模型分析】流量和互动很强、价格低，但粉丝年龄以18岁以下为主，明显不符35岁+占比硬性要求；且学生人设不符合家长/高知/亲子教育家庭方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>pgy:是17宝宝吖～:12000.0:2500.0:安徽 亳州 谯城区</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>是17宝宝吖～</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/59c1cfc044363b34d2522355?track_id=kolMatch_3cfdb458d996418f8bc47c5fd687ab61&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1-3岁/妈妈/家居家装/母婴/4+/白皮</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>安徽 亳州 谯城区</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>2500</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="n">
+        <v>12000</v>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>母婴、家居家装、萌娃</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="n">
+        <v>52</v>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>若放宽项目条件，仅适合低价母婴测评或家庭学习场景，不适合答疑笔核心投放。</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>【大模型分析】报价低且活跃度尚可，但粉丝年龄已知25-34占比58.9%，基本不满足35岁以上占比&gt;40%的硬性要求；人设偏低幼母婴家居，孩子阶段不符，待补CPC/CPE与搜索推荐占比。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>pgy:赞宝赞宝:26000.0:4200.0:安徽 宿州 埇桥区</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>赞宝赞宝</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/64d06a82000000000b007738?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>3-6岁/妈妈/教育/母婴/2+/教育/教育</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>安徽 宿州 埇桥区</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>4200</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>26000</v>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>母婴、萌娃、家居家装</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="n">
+        <v>51</v>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>如补采后受众年龄达标，可尝试家长陪学/启蒙过渡内容；当前更适合低龄教育品。</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>【大模型分析】低报价、有教育母婴标签和蒲公英链接，但孩子为3-6岁倾向，与项目所需小升初/初高中大孩不符；35+粉丝占比、CPC/CPE、搜索推荐流量待补，城市与高知人设也不占优。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>pgy:思思当妈啦:22000.0:2000.0:广西 桂林 灵川县</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>思思当妈啦</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/5eff548700000000010046ac?track_id=kolMatch_3cfdb458d996418f8bc47c5fd687ab61&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>萌娃/妈妈/母婴/测评/教程/教程</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>广西 桂林 灵川县</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="n">
+        <v>22000</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>母婴、萌娃、美食</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="n">
+        <v>51</v>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>更适合母婴测评或低幼家庭产品，不适合本项目初高中大孩教育决策人群。</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>【大模型分析】报价极低、阅读互动数据强，具备性价比；但粉丝年龄已知25-34占比66.7%，大概率不满足35岁以上占比&gt;40%硬性要求，且人设偏育婴师/低幼母婴，孩子阶段明显不符。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>pgy:怂怂:65000.0:3500.0:广东 广州 黄埔区</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>怂怂</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/5f1197ff000000000100600f?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>学生/教育/教程/2+/教育/教育</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>广东 广州 黄埔区</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>3500</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>65000</v>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>教育、娱乐、生活记录</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="n">
+        <v>50</v>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>更适合学生端学习工具传播，不适合本项目以家长为核心的转化链路。</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>【大模型分析】教育教程属性和流量表现不错，报价也可控；但粉丝年龄18-24占比过高，不满足35岁+核心家长画像硬性要求，且学生人设与项目家庭决策场景不符。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>pgy:全能麻麻育儿:25000.0:2000.0:广东 揭阳 榕城区</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>全能麻麻育儿</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/63c2bed40000000026005069?track_id=kolMatch_974f336064d54e6dba74a1521927df82&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1-3岁/妈妈/教育/母婴/2+/教育/教育</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>广东 揭阳 榕城区</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="n">
+        <v>25000</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>母婴、萌娃、家居家装</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="n">
+        <v>38</v>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>待审核</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>不建议进入本项目；如做其他母婴低龄产品，可走性价比测评/教程种草路线。</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>【大模型分析】报价极低且有教育母婴标签、蒲公英链接，但孩子为1-3岁明显不符项目大孩阶段；近30日阅读/曝光表现很弱，流量质量偏差。35+粉丝占比、CPC/CPE、搜索推荐占比仍待补。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>pgy:陈耳东的装修日记:26000.0:4500.0:河南 信阳 息县</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>陈耳东的装修日记</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://pgy.xiaohongshu.com/solar/pre-trade/blogger-detail/657d65ce000000001c019ca7?track_id=kolMatch_3cfdb458d996418f8bc47c5fd687ab61&amp;fromRoute=Advertiser_Kol&amp;source=Advertiser_Kol</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>家居家装/测评</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>河南 信阳 息县</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>4500</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="n">
+        <v>26000</v>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>32%</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>家居家装、美食、生活记录</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="n">
+        <v>28</v>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>不推荐</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>观察暂缓</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>已驳回</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>不建议本项目合作；若跨品类测试，仅可做家庭学习空间/书桌场景软植入。</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>【大模型分析】报价合规且有蒲公英链接，但35岁以上粉丝占比32.4%低于硬门槛40%，且家居装修人设与教育/亲子大孩项目不符；CPC/CPE、搜索推荐占比、孩子阶段待补。</t>
         </is>
       </c>
     </row>

</xml_diff>